<commit_message>
Add whole-workspace export ingestion with individual-file precedence
- parser.py: format detection (workspace/form/workflow), GUID-based
  workspace-export parsing, baseline + surgical-override merge with
  rebuild-time shadow warnings
- Subform role for embedded grids with parent containment edges
- Disabled workflows surfaced: Status column in Excel, dimmed (off)
  nodes + badge in both explorers
- Capture form Description, AutoIncrement fields, duplicate-response
  rules, saved-filter names
- First workspace-export workspace: sce-be (SCE - Building
  Electrification, 36 forms, 22 workflows)
- Document both ingestion formats and the precedence rule in
  CLAUDE.md and README.md

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/global/cross-workspace-inventory.xlsx
+++ b/output/global/cross-workspace-inventory.xlsx
@@ -15,9 +15,11 @@
     <sheet name="DuplicateFlows" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workspaces'!$A$3:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AllForms'!$A$3:$E$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AllWorkflows'!$A$3:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workspaces'!$A$3:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AllForms'!$A$3:$E$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AllWorkflows'!$A$3:$H$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'FormNameCollisions'!$A$3:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DuplicateFlows'!$A$3:$D$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -584,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -669,29 +671,53 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>SCE - Building Electrification</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>1578</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
           <t>socal-whp</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>SCE - ESA Whole Home (PP/D)</t>
         </is>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C6" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D6" s="9" t="n">
         <v>2296</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E6" s="9" t="n">
         <v>48</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F6" s="9" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F5"/>
+  <autoFilter ref="A3:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -702,7 +728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -776,12 +802,12 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>300 - Account Management</t>
+          <t>200 - Account</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -790,173 +816,173 @@
         </is>
       </c>
       <c r="D5" s="9" t="n">
-        <v>353</v>
+        <v>235</v>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>so_cal-esa_whole_home_pp_d__300-account_management_v342_design.json</t>
+          <t>sce-building_electrification.json</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>310 - Enrollment Intake</t>
+          <t>ContactAttemptsGrid</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Spoke</t>
+          <t>Subform</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>161</v>
+        <v>3</v>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>so_cal-esa_whole_home_pp_d__310-enrollment_intake_v97_design.json</t>
+          <t>sce-building_electrification.json</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>315 - SoCal WHP Assessment</t>
+          <t>NotesTable</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Spoke</t>
+          <t>Subform</t>
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>585</v>
+        <v>4</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>so_cal-esa_whole_home_pp_d__315-so_cal_whp_assessment_v105_design.json</t>
+          <t>sce-building_electrification.json</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>325 - SoCal Installation</t>
+          <t>HouseholdMemberInformation</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Spoke</t>
+          <t>Subform</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
-        <v>814</v>
+        <v>6</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>so_cal-esa_whole_home_pp_d__325-so_cal_installation_v92_design.json</t>
+          <t>sce-building_electrification.json</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>395 - Inspection Work Order</t>
+          <t>CampaignDetails</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Spoke</t>
+          <t>Subform</t>
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>134</v>
+        <v>6</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>so_cal-esa_whole_home_pp_d__395-inspection_work_order_v77_design__1_.json</t>
+          <t>sce-building_electrification.json</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>399 - Measures</t>
+          <t>Climate Zones</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Spoke</t>
+          <t>Lookup</t>
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>so_cal-esa_whole_home_pp_d__399-measures_v28_design.json</t>
+          <t>sce-building_electrification.json</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Fee Schedule</t>
+          <t>210 - Enrollment &amp; Assessment Form</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Lookup</t>
+          <t>Spoke</t>
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>23</v>
+        <v>336</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>so_cal-esa_whole_home_pp_d__fee_schedule_v9_design.json</t>
+          <t>sce-building_electrification.json</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>socal-whp</t>
+          <t>sce-be</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>255 - BE Installation Form</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -965,41 +991,941 @@
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>172</v>
+        <v>651</v>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>so_cal-esa_whole_home_pp_d__invoice_v169_design__1_.json</t>
+          <t>sce-building_electrification.json</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>HouseholdMemberInformation (210 - Enrollment &amp; Assessment Form)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>RoomACGrid</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>CorrectionNotesGrid</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>ScopeOfWorkGrid</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>InsulationGrid</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>InstalledInsulation</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>PermitInformation</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>ExistingRoomAC</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>ExistingEVAPCoolerGrid</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>ExistingThermostat</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>NewThermostatInformation</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>ExistingMiniSplitSystem</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>NewMiniSplitSystem</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>NewSystemHeadUnitInformation</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>AlarmDetailGrid</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>CorrectioNotes</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>MinorHomeRepairGrid</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>AdditionalPhotosGrid</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Census Tract</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Lookup</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Spoke</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>131</v>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Fee Schedule</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Lookup</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>InvoiceDetails</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>FinalInvoiceMeasures</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>DownPaymentReviewGrid</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>InvoiceNoteGrid</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Lookup</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>AmendmentsGrid</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>AdjustmentGrid</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Subform</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>sce-building_electrification.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
           <t>socal-whp</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>300 - Account Management</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Hub</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="n">
+        <v>353</v>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>so_cal-esa_whole_home_pp_d__300-account_management_v342_design.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>310 - Enrollment Intake</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Spoke</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>161</v>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>so_cal-esa_whole_home_pp_d__310-enrollment_intake_v97_design.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>315 - SoCal WHP Assessment</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Spoke</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="n">
+        <v>585</v>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>so_cal-esa_whole_home_pp_d__315-so_cal_whp_assessment_v105_design.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>325 - SoCal Installation</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Spoke</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>814</v>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>so_cal-esa_whole_home_pp_d__325-so_cal_installation_v92_design.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>395 - Inspection Work Order</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Spoke</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="n">
+        <v>134</v>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>so_cal-esa_whole_home_pp_d__395-inspection_work_order_v77_design__1_.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>399 - Measures</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Spoke</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>so_cal-esa_whole_home_pp_d__399-measures_v28_design.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Fee Schedule</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Lookup</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>so_cal-esa_whole_home_pp_d__fee_schedule_v9_design.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Spoke</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>172</v>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>so_cal-esa_whole_home_pp_d__invoice_v169_design__1_.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>socal-whp</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
         <is>
           <t>Climate Zones</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C49" s="9" t="inlineStr">
         <is>
           <t>Lookup</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D49" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr">
         <is>
           <t>(no JSON)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E13"/>
+  <autoFilter ref="A3:E49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1010,16 +1936,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1047,20 +1974,25 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
           <t>TriggerForm</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>TriggerAction</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>TargetForms</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Writes</t>
         </is>
@@ -1084,20 +2016,25 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
+          <t>Active/Disabled</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
           <t>Form that fires it</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Create/Update/Delete</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Forms it writes</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Field writes</t>
         </is>
@@ -1106,40 +2043,829 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>CUSTOMER_INT</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Customer Interest Receipt</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>200 - Account</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr"/>
+      <c r="H5" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>APPROVAL_NOT</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Approval Notice Issue</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>200 - Account</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>DESKTOP_REVI</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Desktop Review</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>210 - Enrollment &amp; Assessment Form</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>ENROLLMENT_A</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Enrollment Approved</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>210 - Enrollment &amp; Assessment Form</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>REQUIRES_COR</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Requires Corrections</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>210 - Enrollment &amp; Assessment Form</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>PENDING_REVI</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Pending Reviews</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>210 - Enrollment &amp; Assessment Form</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>RESUBMISSION</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Resubmission for Corrections</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>210 - Enrollment &amp; Assessment Form</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>REVIEW_NOTIF</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Review Notification (Operations)</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>210 - Enrollment &amp; Assessment Form</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>INSTALLATION</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Installation Desktop Review</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>255 - BE Installation Form</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr"/>
+      <c r="H13" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>INSTALLATION_2</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Installation Approved</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>255 - BE Installation Form</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr"/>
+      <c r="H14" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>INSTALLATION_3</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Installation Requires Corrections</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>255 - BE Installation Form</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>PENDING_REVI_2</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Pending Reviews</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>255 - BE Installation Form</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr"/>
+      <c r="G16" s="9" t="inlineStr"/>
+      <c r="H16" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>REVIEW_NOTIF_2</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Review Notification (Operations)</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>255 - BE Installation Form</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr"/>
+      <c r="H17" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>INVOICE_SUBM</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Invoice Submitted by Contractor - Final</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr"/>
+      <c r="H18" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>INVOICE_SUBM_2</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Invoice Submitted by Contractor - Down Payment</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr"/>
+      <c r="H19" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>APPROVED_BY_</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Approved by Coordinator - Down Payment</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr"/>
+      <c r="H20" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>APPROVED_BY__2</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Approved by PM - Down Payment</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr"/>
+      <c r="H21" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>APPROVED_BY__3</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Approved by PM - Final Invoice</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr"/>
+      <c r="H22" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>CORRECTIONS_</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Corrections Required - Down Payment</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr"/>
+      <c r="H23" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>INVOICE_REJE</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Invoice Rejected by Management - Final</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr"/>
+      <c r="H24" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>CORRECTIONS__2</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Corrections Required - Final</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr"/>
+      <c r="H25" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>REVIEW_NOTIF_3</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Review Notification (Operations)</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Update</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr"/>
+      <c r="H26" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
           <t>socal-whp</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>INSPECT-01</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>Create Inspection</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>300 - Account Management</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>395 - Inspection Work Order</t>
         </is>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="H27" s="9" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:G5"/>
+  <autoFilter ref="A3:H27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1150,7 +2876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1210,7 +2936,68 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Climate Zones</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>sce-be, socal-whp</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Fee Schedule</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>sce-be, socal-whp</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>sce-be, socal-whp</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Spoke</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A3:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1221,7 +3008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -1281,7 +3068,68 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Update -&gt; (no target)</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>sce-be/APPROVAL_NOT, sce-be/DESKTOP_REVI, sce-be/ENROLLMENT_A, sce-be/REQUIRES_COR, sce-be/RESUBMISSION, sce-be/REVIEW_NOTIF, sce-be/INSTALLATION, sce-be/INSTALLATION_2, sce-be/INSTALLATION_3, sce-be/REVIEW_NOTIF_2, sce-be/INVOICE_SUBM, sce-be/APPROVED_BY_, sce-be/APPROVED_BY__2, sce-be/APPROVED_BY__3, sce-be/CORRECTIONS_, sce-be/INVOICE_REJE, sce-be/CORRECTIONS__2, sce-be/REVIEW_NOTIF_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>(none) -&gt; (no target)</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>sce-be/PENDING_REVI, sce-be/PENDING_REVI_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Create -&gt; (no target)</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>sce-be</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>sce-be/CUSTOMER_INT, sce-be/INVOICE_SUBM_2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A3:D7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: harden explorers and generated inventory
</commit_message>
<xml_diff>
--- a/output/global/cross-workspace-inventory.xlsx
+++ b/output/global/cross-workspace-inventory.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AllForms" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AllWorkflows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FormNameCollisions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DuplicateFlows" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowReuse" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FormFamilies" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldTemplates" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Workspaces" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="AllForms" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="AllWorkflows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="FormNameCollisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DuplicateFlows" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="WorkflowReuse" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="FormFamilies" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="FieldTemplates" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workspaces'!$A$3:$F$9</definedName>

</xml_diff>